<commit_message>
三大法人更新 2026/05/03 14:57 UTC
</commit_message>
<xml_diff>
--- a/cb_inst_20260430.xlsx
+++ b/cb_inst_20260430.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -47,7 +44,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,21 +52,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -457,72 +445,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CB代號</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>CB名稱</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>外資_買張</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>外資_賣張</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>外資_買賣超</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>投信_買張</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>投信_賣張</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>投信_買賣超</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>自營_買張</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>自營_賣張</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>自營_買賣超</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>三大法人合計買賣超</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>買超方向</t>
         </is>
@@ -571,7 +559,7 @@
       <c r="L2" t="n">
         <v>200</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="M2" s="1" t="n">
         <v>200</v>
       </c>
       <c r="N2" t="inlineStr">
@@ -623,7 +611,7 @@
       <c r="L3" t="n">
         <v>-35</v>
       </c>
-      <c r="M3" s="2" t="n">
+      <c r="M3" s="1" t="n">
         <v>115</v>
       </c>
       <c r="N3" t="inlineStr">
@@ -675,7 +663,7 @@
       <c r="L4" t="n">
         <v>99</v>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="M4" s="1" t="n">
         <v>99</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -727,7 +715,7 @@
       <c r="L5" t="n">
         <v>96</v>
       </c>
-      <c r="M5" s="2" t="n">
+      <c r="M5" s="1" t="n">
         <v>96</v>
       </c>
       <c r="N5" t="inlineStr">
@@ -779,7 +767,7 @@
       <c r="L6" t="n">
         <v>52</v>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="1" t="n">
         <v>52</v>
       </c>
       <c r="N6" t="inlineStr">
@@ -831,7 +819,7 @@
       <c r="L7" t="n">
         <v>27</v>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="1" t="n">
         <v>50</v>
       </c>
       <c r="N7" t="inlineStr">
@@ -883,7 +871,7 @@
       <c r="L8" t="n">
         <v>49</v>
       </c>
-      <c r="M8" s="2" t="n">
+      <c r="M8" s="1" t="n">
         <v>49</v>
       </c>
       <c r="N8" t="inlineStr">
@@ -935,7 +923,7 @@
       <c r="L9" t="n">
         <v>37</v>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" s="1" t="n">
         <v>37</v>
       </c>
       <c r="N9" t="inlineStr">
@@ -987,7 +975,7 @@
       <c r="L10" t="n">
         <v>102</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="1" t="n">
         <v>37</v>
       </c>
       <c r="N10" t="inlineStr">
@@ -1039,7 +1027,7 @@
       <c r="L11" t="n">
         <v>37</v>
       </c>
-      <c r="M11" s="2" t="n">
+      <c r="M11" s="1" t="n">
         <v>37</v>
       </c>
       <c r="N11" t="inlineStr">
@@ -1091,7 +1079,7 @@
       <c r="L12" t="n">
         <v>35</v>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="M12" s="1" t="n">
         <v>35</v>
       </c>
       <c r="N12" t="inlineStr">
@@ -1143,7 +1131,7 @@
       <c r="L13" t="n">
         <v>-20</v>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M13" s="1" t="n">
         <v>35</v>
       </c>
       <c r="N13" t="inlineStr">
@@ -1195,7 +1183,7 @@
       <c r="L14" t="n">
         <v>34</v>
       </c>
-      <c r="M14" s="2" t="n">
+      <c r="M14" s="1" t="n">
         <v>34</v>
       </c>
       <c r="N14" t="inlineStr">
@@ -1247,7 +1235,7 @@
       <c r="L15" t="n">
         <v>33</v>
       </c>
-      <c r="M15" s="2" t="n">
+      <c r="M15" s="1" t="n">
         <v>33</v>
       </c>
       <c r="N15" t="inlineStr">
@@ -1299,7 +1287,7 @@
       <c r="L16" t="n">
         <v>33</v>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="M16" s="1" t="n">
         <v>33</v>
       </c>
       <c r="N16" t="inlineStr">
@@ -1351,7 +1339,7 @@
       <c r="L17" t="n">
         <v>2</v>
       </c>
-      <c r="M17" s="2" t="n">
+      <c r="M17" s="1" t="n">
         <v>32</v>
       </c>
       <c r="N17" t="inlineStr">
@@ -1403,7 +1391,7 @@
       <c r="L18" t="n">
         <v>32</v>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="M18" s="1" t="n">
         <v>32</v>
       </c>
       <c r="N18" t="inlineStr">
@@ -1455,7 +1443,7 @@
       <c r="L19" t="n">
         <v>28</v>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="M19" s="1" t="n">
         <v>28</v>
       </c>
       <c r="N19" t="inlineStr">
@@ -1507,7 +1495,7 @@
       <c r="L20" t="n">
         <v>20</v>
       </c>
-      <c r="M20" s="2" t="n">
+      <c r="M20" s="1" t="n">
         <v>20</v>
       </c>
       <c r="N20" t="inlineStr">
@@ -1559,7 +1547,7 @@
       <c r="L21" t="n">
         <v>20</v>
       </c>
-      <c r="M21" s="2" t="n">
+      <c r="M21" s="1" t="n">
         <v>20</v>
       </c>
       <c r="N21" t="inlineStr">
@@ -1611,7 +1599,7 @@
       <c r="L22" t="n">
         <v>20</v>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="M22" s="1" t="n">
         <v>20</v>
       </c>
       <c r="N22" t="inlineStr">
@@ -1663,7 +1651,7 @@
       <c r="L23" t="n">
         <v>20</v>
       </c>
-      <c r="M23" s="2" t="n">
+      <c r="M23" s="1" t="n">
         <v>20</v>
       </c>
       <c r="N23" t="inlineStr">
@@ -1715,7 +1703,7 @@
       <c r="L24" t="n">
         <v>19</v>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="M24" s="1" t="n">
         <v>19</v>
       </c>
       <c r="N24" t="inlineStr">
@@ -1767,7 +1755,7 @@
       <c r="L25" t="n">
         <v>19</v>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="M25" s="1" t="n">
         <v>19</v>
       </c>
       <c r="N25" t="inlineStr">
@@ -1819,7 +1807,7 @@
       <c r="L26" t="n">
         <v>19</v>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="M26" s="1" t="n">
         <v>19</v>
       </c>
       <c r="N26" t="inlineStr">
@@ -1871,7 +1859,7 @@
       <c r="L27" t="n">
         <v>16</v>
       </c>
-      <c r="M27" s="2" t="n">
+      <c r="M27" s="1" t="n">
         <v>16</v>
       </c>
       <c r="N27" t="inlineStr">
@@ -1923,7 +1911,7 @@
       <c r="L28" t="n">
         <v>15</v>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="M28" s="1" t="n">
         <v>15</v>
       </c>
       <c r="N28" t="inlineStr">
@@ -1975,7 +1963,7 @@
       <c r="L29" t="n">
         <v>15</v>
       </c>
-      <c r="M29" s="2" t="n">
+      <c r="M29" s="1" t="n">
         <v>15</v>
       </c>
       <c r="N29" t="inlineStr">
@@ -2027,7 +2015,7 @@
       <c r="L30" t="n">
         <v>14</v>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="M30" s="1" t="n">
         <v>14</v>
       </c>
       <c r="N30" t="inlineStr">
@@ -2079,7 +2067,7 @@
       <c r="L31" t="n">
         <v>22</v>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="M31" s="1" t="n">
         <v>14</v>
       </c>
       <c r="N31" t="inlineStr">
@@ -2131,7 +2119,7 @@
       <c r="L32" t="n">
         <v>13</v>
       </c>
-      <c r="M32" s="2" t="n">
+      <c r="M32" s="1" t="n">
         <v>13</v>
       </c>
       <c r="N32" t="inlineStr">
@@ -2183,7 +2171,7 @@
       <c r="L33" t="n">
         <v>12</v>
       </c>
-      <c r="M33" s="2" t="n">
+      <c r="M33" s="1" t="n">
         <v>12</v>
       </c>
       <c r="N33" t="inlineStr">
@@ -2235,7 +2223,7 @@
       <c r="L34" t="n">
         <v>12</v>
       </c>
-      <c r="M34" s="2" t="n">
+      <c r="M34" s="1" t="n">
         <v>12</v>
       </c>
       <c r="N34" t="inlineStr">
@@ -2287,7 +2275,7 @@
       <c r="L35" t="n">
         <v>11</v>
       </c>
-      <c r="M35" s="2" t="n">
+      <c r="M35" s="1" t="n">
         <v>11</v>
       </c>
       <c r="N35" t="inlineStr">
@@ -2339,7 +2327,7 @@
       <c r="L36" t="n">
         <v>11</v>
       </c>
-      <c r="M36" s="2" t="n">
+      <c r="M36" s="1" t="n">
         <v>11</v>
       </c>
       <c r="N36" t="inlineStr">
@@ -2391,7 +2379,7 @@
       <c r="L37" t="n">
         <v>10</v>
       </c>
-      <c r="M37" s="2" t="n">
+      <c r="M37" s="1" t="n">
         <v>10</v>
       </c>
       <c r="N37" t="inlineStr">
@@ -2443,7 +2431,7 @@
       <c r="L38" t="n">
         <v>9</v>
       </c>
-      <c r="M38" s="2" t="n">
+      <c r="M38" s="1" t="n">
         <v>9</v>
       </c>
       <c r="N38" t="inlineStr">
@@ -2495,7 +2483,7 @@
       <c r="L39" t="n">
         <v>9</v>
       </c>
-      <c r="M39" s="2" t="n">
+      <c r="M39" s="1" t="n">
         <v>9</v>
       </c>
       <c r="N39" t="inlineStr">
@@ -2547,7 +2535,7 @@
       <c r="L40" t="n">
         <v>7</v>
       </c>
-      <c r="M40" s="2" t="n">
+      <c r="M40" s="1" t="n">
         <v>7</v>
       </c>
       <c r="N40" t="inlineStr">
@@ -2599,7 +2587,7 @@
       <c r="L41" t="n">
         <v>7</v>
       </c>
-      <c r="M41" s="2" t="n">
+      <c r="M41" s="1" t="n">
         <v>7</v>
       </c>
       <c r="N41" t="inlineStr">
@@ -2651,7 +2639,7 @@
       <c r="L42" t="n">
         <v>7</v>
       </c>
-      <c r="M42" s="2" t="n">
+      <c r="M42" s="1" t="n">
         <v>7</v>
       </c>
       <c r="N42" t="inlineStr">
@@ -2703,7 +2691,7 @@
       <c r="L43" t="n">
         <v>7</v>
       </c>
-      <c r="M43" s="2" t="n">
+      <c r="M43" s="1" t="n">
         <v>7</v>
       </c>
       <c r="N43" t="inlineStr">
@@ -2755,7 +2743,7 @@
       <c r="L44" t="n">
         <v>6</v>
       </c>
-      <c r="M44" s="2" t="n">
+      <c r="M44" s="1" t="n">
         <v>6</v>
       </c>
       <c r="N44" t="inlineStr">
@@ -2807,7 +2795,7 @@
       <c r="L45" t="n">
         <v>6</v>
       </c>
-      <c r="M45" s="2" t="n">
+      <c r="M45" s="1" t="n">
         <v>6</v>
       </c>
       <c r="N45" t="inlineStr">
@@ -2859,7 +2847,7 @@
       <c r="L46" t="n">
         <v>6</v>
       </c>
-      <c r="M46" s="2" t="n">
+      <c r="M46" s="1" t="n">
         <v>6</v>
       </c>
       <c r="N46" t="inlineStr">
@@ -2911,7 +2899,7 @@
       <c r="L47" t="n">
         <v>6</v>
       </c>
-      <c r="M47" s="2" t="n">
+      <c r="M47" s="1" t="n">
         <v>6</v>
       </c>
       <c r="N47" t="inlineStr">
@@ -2963,7 +2951,7 @@
       <c r="L48" t="n">
         <v>5</v>
       </c>
-      <c r="M48" s="2" t="n">
+      <c r="M48" s="1" t="n">
         <v>5</v>
       </c>
       <c r="N48" t="inlineStr">
@@ -3015,7 +3003,7 @@
       <c r="L49" t="n">
         <v>5</v>
       </c>
-      <c r="M49" s="2" t="n">
+      <c r="M49" s="1" t="n">
         <v>5</v>
       </c>
       <c r="N49" t="inlineStr">
@@ -3067,7 +3055,7 @@
       <c r="L50" t="n">
         <v>5</v>
       </c>
-      <c r="M50" s="2" t="n">
+      <c r="M50" s="1" t="n">
         <v>5</v>
       </c>
       <c r="N50" t="inlineStr">
@@ -3119,7 +3107,7 @@
       <c r="L51" t="n">
         <v>4</v>
       </c>
-      <c r="M51" s="2" t="n">
+      <c r="M51" s="1" t="n">
         <v>4</v>
       </c>
       <c r="N51" t="inlineStr">
@@ -3171,7 +3159,7 @@
       <c r="L52" t="n">
         <v>4</v>
       </c>
-      <c r="M52" s="2" t="n">
+      <c r="M52" s="1" t="n">
         <v>4</v>
       </c>
       <c r="N52" t="inlineStr">
@@ -3223,7 +3211,7 @@
       <c r="L53" t="n">
         <v>4</v>
       </c>
-      <c r="M53" s="2" t="n">
+      <c r="M53" s="1" t="n">
         <v>4</v>
       </c>
       <c r="N53" t="inlineStr">
@@ -3275,7 +3263,7 @@
       <c r="L54" t="n">
         <v>3</v>
       </c>
-      <c r="M54" s="2" t="n">
+      <c r="M54" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N54" t="inlineStr">
@@ -3327,7 +3315,7 @@
       <c r="L55" t="n">
         <v>3</v>
       </c>
-      <c r="M55" s="2" t="n">
+      <c r="M55" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N55" t="inlineStr">
@@ -3379,7 +3367,7 @@
       <c r="L56" t="n">
         <v>3</v>
       </c>
-      <c r="M56" s="2" t="n">
+      <c r="M56" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N56" t="inlineStr">
@@ -3431,7 +3419,7 @@
       <c r="L57" t="n">
         <v>3</v>
       </c>
-      <c r="M57" s="2" t="n">
+      <c r="M57" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N57" t="inlineStr">
@@ -3483,7 +3471,7 @@
       <c r="L58" t="n">
         <v>3</v>
       </c>
-      <c r="M58" s="2" t="n">
+      <c r="M58" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N58" t="inlineStr">
@@ -3535,7 +3523,7 @@
       <c r="L59" t="n">
         <v>3</v>
       </c>
-      <c r="M59" s="2" t="n">
+      <c r="M59" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N59" t="inlineStr">
@@ -3587,7 +3575,7 @@
       <c r="L60" t="n">
         <v>3</v>
       </c>
-      <c r="M60" s="2" t="n">
+      <c r="M60" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N60" t="inlineStr">
@@ -3639,7 +3627,7 @@
       <c r="L61" t="n">
         <v>3</v>
       </c>
-      <c r="M61" s="2" t="n">
+      <c r="M61" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N61" t="inlineStr">
@@ -3691,7 +3679,7 @@
       <c r="L62" t="n">
         <v>13</v>
       </c>
-      <c r="M62" s="2" t="n">
+      <c r="M62" s="1" t="n">
         <v>3</v>
       </c>
       <c r="N62" t="inlineStr">
@@ -3743,7 +3731,7 @@
       <c r="L63" t="n">
         <v>2</v>
       </c>
-      <c r="M63" s="2" t="n">
+      <c r="M63" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N63" t="inlineStr">
@@ -3795,7 +3783,7 @@
       <c r="L64" t="n">
         <v>2</v>
       </c>
-      <c r="M64" s="2" t="n">
+      <c r="M64" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N64" t="inlineStr">
@@ -3847,7 +3835,7 @@
       <c r="L65" t="n">
         <v>2</v>
       </c>
-      <c r="M65" s="2" t="n">
+      <c r="M65" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N65" t="inlineStr">
@@ -3899,7 +3887,7 @@
       <c r="L66" t="n">
         <v>2</v>
       </c>
-      <c r="M66" s="2" t="n">
+      <c r="M66" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N66" t="inlineStr">
@@ -3951,7 +3939,7 @@
       <c r="L67" t="n">
         <v>2</v>
       </c>
-      <c r="M67" s="2" t="n">
+      <c r="M67" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N67" t="inlineStr">
@@ -4003,7 +3991,7 @@
       <c r="L68" t="n">
         <v>2</v>
       </c>
-      <c r="M68" s="2" t="n">
+      <c r="M68" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N68" t="inlineStr">
@@ -4055,7 +4043,7 @@
       <c r="L69" t="n">
         <v>2</v>
       </c>
-      <c r="M69" s="2" t="n">
+      <c r="M69" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N69" t="inlineStr">
@@ -4107,7 +4095,7 @@
       <c r="L70" t="n">
         <v>2</v>
       </c>
-      <c r="M70" s="2" t="n">
+      <c r="M70" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N70" t="inlineStr">
@@ -4159,7 +4147,7 @@
       <c r="L71" t="n">
         <v>2</v>
       </c>
-      <c r="M71" s="2" t="n">
+      <c r="M71" s="1" t="n">
         <v>2</v>
       </c>
       <c r="N71" t="inlineStr">
@@ -4211,7 +4199,7 @@
       <c r="L72" t="n">
         <v>14</v>
       </c>
-      <c r="M72" s="2" t="n">
+      <c r="M72" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N72" t="inlineStr">
@@ -4263,7 +4251,7 @@
       <c r="L73" t="n">
         <v>1</v>
       </c>
-      <c r="M73" s="2" t="n">
+      <c r="M73" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N73" t="inlineStr">
@@ -4315,7 +4303,7 @@
       <c r="L74" t="n">
         <v>1</v>
       </c>
-      <c r="M74" s="2" t="n">
+      <c r="M74" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N74" t="inlineStr">
@@ -4367,7 +4355,7 @@
       <c r="L75" t="n">
         <v>1</v>
       </c>
-      <c r="M75" s="2" t="n">
+      <c r="M75" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N75" t="inlineStr">
@@ -4419,7 +4407,7 @@
       <c r="L76" t="n">
         <v>1</v>
       </c>
-      <c r="M76" s="2" t="n">
+      <c r="M76" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N76" t="inlineStr">
@@ -4471,7 +4459,7 @@
       <c r="L77" t="n">
         <v>1</v>
       </c>
-      <c r="M77" s="2" t="n">
+      <c r="M77" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N77" t="inlineStr">
@@ -4523,7 +4511,7 @@
       <c r="L78" t="n">
         <v>1</v>
       </c>
-      <c r="M78" s="2" t="n">
+      <c r="M78" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N78" t="inlineStr">
@@ -4575,7 +4563,7 @@
       <c r="L79" t="n">
         <v>1</v>
       </c>
-      <c r="M79" s="2" t="n">
+      <c r="M79" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N79" t="inlineStr">
@@ -4627,7 +4615,7 @@
       <c r="L80" t="n">
         <v>1</v>
       </c>
-      <c r="M80" s="2" t="n">
+      <c r="M80" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N80" t="inlineStr">
@@ -4679,7 +4667,7 @@
       <c r="L81" t="n">
         <v>1</v>
       </c>
-      <c r="M81" s="2" t="n">
+      <c r="M81" s="1" t="n">
         <v>1</v>
       </c>
       <c r="N81" t="inlineStr">
@@ -6135,7 +6123,7 @@
       <c r="L109" t="n">
         <v>-1</v>
       </c>
-      <c r="M109" s="3" t="n">
+      <c r="M109" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N109" t="inlineStr">
@@ -6187,7 +6175,7 @@
       <c r="L110" t="n">
         <v>-1</v>
       </c>
-      <c r="M110" s="3" t="n">
+      <c r="M110" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N110" t="inlineStr">
@@ -6239,7 +6227,7 @@
       <c r="L111" t="n">
         <v>-1</v>
       </c>
-      <c r="M111" s="3" t="n">
+      <c r="M111" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N111" t="inlineStr">
@@ -6291,7 +6279,7 @@
       <c r="L112" t="n">
         <v>-1</v>
       </c>
-      <c r="M112" s="3" t="n">
+      <c r="M112" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N112" t="inlineStr">
@@ -6343,7 +6331,7 @@
       <c r="L113" t="n">
         <v>-1</v>
       </c>
-      <c r="M113" s="3" t="n">
+      <c r="M113" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N113" t="inlineStr">
@@ -6395,7 +6383,7 @@
       <c r="L114" t="n">
         <v>-1</v>
       </c>
-      <c r="M114" s="3" t="n">
+      <c r="M114" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N114" t="inlineStr">
@@ -6447,7 +6435,7 @@
       <c r="L115" t="n">
         <v>-1</v>
       </c>
-      <c r="M115" s="3" t="n">
+      <c r="M115" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N115" t="inlineStr">
@@ -6499,7 +6487,7 @@
       <c r="L116" t="n">
         <v>-1</v>
       </c>
-      <c r="M116" s="3" t="n">
+      <c r="M116" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N116" t="inlineStr">
@@ -6551,7 +6539,7 @@
       <c r="L117" t="n">
         <v>-1</v>
       </c>
-      <c r="M117" s="3" t="n">
+      <c r="M117" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N117" t="inlineStr">
@@ -6603,7 +6591,7 @@
       <c r="L118" t="n">
         <v>-2</v>
       </c>
-      <c r="M118" s="3" t="n">
+      <c r="M118" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N118" t="inlineStr">
@@ -6655,7 +6643,7 @@
       <c r="L119" t="n">
         <v>-2</v>
       </c>
-      <c r="M119" s="3" t="n">
+      <c r="M119" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N119" t="inlineStr">
@@ -6707,7 +6695,7 @@
       <c r="L120" t="n">
         <v>-2</v>
       </c>
-      <c r="M120" s="3" t="n">
+      <c r="M120" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N120" t="inlineStr">
@@ -6759,7 +6747,7 @@
       <c r="L121" t="n">
         <v>-2</v>
       </c>
-      <c r="M121" s="3" t="n">
+      <c r="M121" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N121" t="inlineStr">
@@ -6811,7 +6799,7 @@
       <c r="L122" t="n">
         <v>-2</v>
       </c>
-      <c r="M122" s="3" t="n">
+      <c r="M122" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N122" t="inlineStr">
@@ -6863,7 +6851,7 @@
       <c r="L123" t="n">
         <v>-2</v>
       </c>
-      <c r="M123" s="3" t="n">
+      <c r="M123" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N123" t="inlineStr">
@@ -6915,7 +6903,7 @@
       <c r="L124" t="n">
         <v>-2</v>
       </c>
-      <c r="M124" s="3" t="n">
+      <c r="M124" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N124" t="inlineStr">
@@ -6967,7 +6955,7 @@
       <c r="L125" t="n">
         <v>-2</v>
       </c>
-      <c r="M125" s="3" t="n">
+      <c r="M125" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N125" t="inlineStr">
@@ -7019,7 +7007,7 @@
       <c r="L126" t="n">
         <v>-2</v>
       </c>
-      <c r="M126" s="3" t="n">
+      <c r="M126" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N126" t="inlineStr">
@@ -7071,7 +7059,7 @@
       <c r="L127" t="n">
         <v>-2</v>
       </c>
-      <c r="M127" s="3" t="n">
+      <c r="M127" s="2" t="n">
         <v>-2</v>
       </c>
       <c r="N127" t="inlineStr">
@@ -7123,7 +7111,7 @@
       <c r="L128" t="n">
         <v>-3</v>
       </c>
-      <c r="M128" s="3" t="n">
+      <c r="M128" s="2" t="n">
         <v>-3</v>
       </c>
       <c r="N128" t="inlineStr">
@@ -7175,7 +7163,7 @@
       <c r="L129" t="n">
         <v>-3</v>
       </c>
-      <c r="M129" s="3" t="n">
+      <c r="M129" s="2" t="n">
         <v>-3</v>
       </c>
       <c r="N129" t="inlineStr">
@@ -7227,7 +7215,7 @@
       <c r="L130" t="n">
         <v>-3</v>
       </c>
-      <c r="M130" s="3" t="n">
+      <c r="M130" s="2" t="n">
         <v>-3</v>
       </c>
       <c r="N130" t="inlineStr">
@@ -7279,7 +7267,7 @@
       <c r="L131" t="n">
         <v>-4</v>
       </c>
-      <c r="M131" s="3" t="n">
+      <c r="M131" s="2" t="n">
         <v>-4</v>
       </c>
       <c r="N131" t="inlineStr">
@@ -7331,7 +7319,7 @@
       <c r="L132" t="n">
         <v>-4</v>
       </c>
-      <c r="M132" s="3" t="n">
+      <c r="M132" s="2" t="n">
         <v>-4</v>
       </c>
       <c r="N132" t="inlineStr">
@@ -7383,7 +7371,7 @@
       <c r="L133" t="n">
         <v>-4</v>
       </c>
-      <c r="M133" s="3" t="n">
+      <c r="M133" s="2" t="n">
         <v>-4</v>
       </c>
       <c r="N133" t="inlineStr">
@@ -7435,7 +7423,7 @@
       <c r="L134" t="n">
         <v>-4</v>
       </c>
-      <c r="M134" s="3" t="n">
+      <c r="M134" s="2" t="n">
         <v>-4</v>
       </c>
       <c r="N134" t="inlineStr">
@@ -7487,7 +7475,7 @@
       <c r="L135" t="n">
         <v>-5</v>
       </c>
-      <c r="M135" s="3" t="n">
+      <c r="M135" s="2" t="n">
         <v>-5</v>
       </c>
       <c r="N135" t="inlineStr">
@@ -7539,7 +7527,7 @@
       <c r="L136" t="n">
         <v>0</v>
       </c>
-      <c r="M136" s="3" t="n">
+      <c r="M136" s="2" t="n">
         <v>-5</v>
       </c>
       <c r="N136" t="inlineStr">
@@ -7591,7 +7579,7 @@
       <c r="L137" t="n">
         <v>-5</v>
       </c>
-      <c r="M137" s="3" t="n">
+      <c r="M137" s="2" t="n">
         <v>-5</v>
       </c>
       <c r="N137" t="inlineStr">
@@ -7643,7 +7631,7 @@
       <c r="L138" t="n">
         <v>-5</v>
       </c>
-      <c r="M138" s="3" t="n">
+      <c r="M138" s="2" t="n">
         <v>-5</v>
       </c>
       <c r="N138" t="inlineStr">
@@ -7695,7 +7683,7 @@
       <c r="L139" t="n">
         <v>-5</v>
       </c>
-      <c r="M139" s="3" t="n">
+      <c r="M139" s="2" t="n">
         <v>-5</v>
       </c>
       <c r="N139" t="inlineStr">
@@ -7747,7 +7735,7 @@
       <c r="L140" t="n">
         <v>-5</v>
       </c>
-      <c r="M140" s="3" t="n">
+      <c r="M140" s="2" t="n">
         <v>-5</v>
       </c>
       <c r="N140" t="inlineStr">
@@ -7799,7 +7787,7 @@
       <c r="L141" t="n">
         <v>-6</v>
       </c>
-      <c r="M141" s="3" t="n">
+      <c r="M141" s="2" t="n">
         <v>-6</v>
       </c>
       <c r="N141" t="inlineStr">
@@ -7851,7 +7839,7 @@
       <c r="L142" t="n">
         <v>-7</v>
       </c>
-      <c r="M142" s="3" t="n">
+      <c r="M142" s="2" t="n">
         <v>-7</v>
       </c>
       <c r="N142" t="inlineStr">
@@ -7903,7 +7891,7 @@
       <c r="L143" t="n">
         <v>-7</v>
       </c>
-      <c r="M143" s="3" t="n">
+      <c r="M143" s="2" t="n">
         <v>-7</v>
       </c>
       <c r="N143" t="inlineStr">
@@ -7955,7 +7943,7 @@
       <c r="L144" t="n">
         <v>-7</v>
       </c>
-      <c r="M144" s="3" t="n">
+      <c r="M144" s="2" t="n">
         <v>-7</v>
       </c>
       <c r="N144" t="inlineStr">
@@ -8007,7 +7995,7 @@
       <c r="L145" t="n">
         <v>-8</v>
       </c>
-      <c r="M145" s="3" t="n">
+      <c r="M145" s="2" t="n">
         <v>-8</v>
       </c>
       <c r="N145" t="inlineStr">
@@ -8059,7 +8047,7 @@
       <c r="L146" t="n">
         <v>-8</v>
       </c>
-      <c r="M146" s="3" t="n">
+      <c r="M146" s="2" t="n">
         <v>-8</v>
       </c>
       <c r="N146" t="inlineStr">
@@ -8111,7 +8099,7 @@
       <c r="L147" t="n">
         <v>-9</v>
       </c>
-      <c r="M147" s="3" t="n">
+      <c r="M147" s="2" t="n">
         <v>-9</v>
       </c>
       <c r="N147" t="inlineStr">
@@ -8163,7 +8151,7 @@
       <c r="L148" t="n">
         <v>-10</v>
       </c>
-      <c r="M148" s="3" t="n">
+      <c r="M148" s="2" t="n">
         <v>-10</v>
       </c>
       <c r="N148" t="inlineStr">
@@ -8215,7 +8203,7 @@
       <c r="L149" t="n">
         <v>-10</v>
       </c>
-      <c r="M149" s="3" t="n">
+      <c r="M149" s="2" t="n">
         <v>-10</v>
       </c>
       <c r="N149" t="inlineStr">
@@ -8267,7 +8255,7 @@
       <c r="L150" t="n">
         <v>-10</v>
       </c>
-      <c r="M150" s="3" t="n">
+      <c r="M150" s="2" t="n">
         <v>-10</v>
       </c>
       <c r="N150" t="inlineStr">
@@ -8319,7 +8307,7 @@
       <c r="L151" t="n">
         <v>-10</v>
       </c>
-      <c r="M151" s="3" t="n">
+      <c r="M151" s="2" t="n">
         <v>-10</v>
       </c>
       <c r="N151" t="inlineStr">
@@ -8371,7 +8359,7 @@
       <c r="L152" t="n">
         <v>-11</v>
       </c>
-      <c r="M152" s="3" t="n">
+      <c r="M152" s="2" t="n">
         <v>-11</v>
       </c>
       <c r="N152" t="inlineStr">
@@ -8423,7 +8411,7 @@
       <c r="L153" t="n">
         <v>0</v>
       </c>
-      <c r="M153" s="3" t="n">
+      <c r="M153" s="2" t="n">
         <v>-12</v>
       </c>
       <c r="N153" t="inlineStr">
@@ -8475,7 +8463,7 @@
       <c r="L154" t="n">
         <v>-12</v>
       </c>
-      <c r="M154" s="3" t="n">
+      <c r="M154" s="2" t="n">
         <v>-12</v>
       </c>
       <c r="N154" t="inlineStr">
@@ -8527,7 +8515,7 @@
       <c r="L155" t="n">
         <v>-12</v>
       </c>
-      <c r="M155" s="3" t="n">
+      <c r="M155" s="2" t="n">
         <v>-12</v>
       </c>
       <c r="N155" t="inlineStr">
@@ -8579,7 +8567,7 @@
       <c r="L156" t="n">
         <v>-2</v>
       </c>
-      <c r="M156" s="3" t="n">
+      <c r="M156" s="2" t="n">
         <v>-12</v>
       </c>
       <c r="N156" t="inlineStr">
@@ -8631,7 +8619,7 @@
       <c r="L157" t="n">
         <v>-13</v>
       </c>
-      <c r="M157" s="3" t="n">
+      <c r="M157" s="2" t="n">
         <v>-13</v>
       </c>
       <c r="N157" t="inlineStr">
@@ -8683,7 +8671,7 @@
       <c r="L158" t="n">
         <v>-14</v>
       </c>
-      <c r="M158" s="3" t="n">
+      <c r="M158" s="2" t="n">
         <v>-14</v>
       </c>
       <c r="N158" t="inlineStr">
@@ -8735,7 +8723,7 @@
       <c r="L159" t="n">
         <v>-16</v>
       </c>
-      <c r="M159" s="3" t="n">
+      <c r="M159" s="2" t="n">
         <v>-16</v>
       </c>
       <c r="N159" t="inlineStr">
@@ -8787,7 +8775,7 @@
       <c r="L160" t="n">
         <v>-20</v>
       </c>
-      <c r="M160" s="3" t="n">
+      <c r="M160" s="2" t="n">
         <v>-20</v>
       </c>
       <c r="N160" t="inlineStr">
@@ -8839,7 +8827,7 @@
       <c r="L161" t="n">
         <v>0</v>
       </c>
-      <c r="M161" s="3" t="n">
+      <c r="M161" s="2" t="n">
         <v>-20</v>
       </c>
       <c r="N161" t="inlineStr">
@@ -8891,7 +8879,7 @@
       <c r="L162" t="n">
         <v>-22</v>
       </c>
-      <c r="M162" s="3" t="n">
+      <c r="M162" s="2" t="n">
         <v>-22</v>
       </c>
       <c r="N162" t="inlineStr">
@@ -8943,7 +8931,7 @@
       <c r="L163" t="n">
         <v>-16</v>
       </c>
-      <c r="M163" s="3" t="n">
+      <c r="M163" s="2" t="n">
         <v>-23</v>
       </c>
       <c r="N163" t="inlineStr">
@@ -8995,7 +8983,7 @@
       <c r="L164" t="n">
         <v>-23</v>
       </c>
-      <c r="M164" s="3" t="n">
+      <c r="M164" s="2" t="n">
         <v>-23</v>
       </c>
       <c r="N164" t="inlineStr">
@@ -9047,7 +9035,7 @@
       <c r="L165" t="n">
         <v>-25</v>
       </c>
-      <c r="M165" s="3" t="n">
+      <c r="M165" s="2" t="n">
         <v>-25</v>
       </c>
       <c r="N165" t="inlineStr">
@@ -9099,7 +9087,7 @@
       <c r="L166" t="n">
         <v>-25</v>
       </c>
-      <c r="M166" s="3" t="n">
+      <c r="M166" s="2" t="n">
         <v>-25</v>
       </c>
       <c r="N166" t="inlineStr">
@@ -9151,7 +9139,7 @@
       <c r="L167" t="n">
         <v>-25</v>
       </c>
-      <c r="M167" s="3" t="n">
+      <c r="M167" s="2" t="n">
         <v>-25</v>
       </c>
       <c r="N167" t="inlineStr">
@@ -9203,7 +9191,7 @@
       <c r="L168" t="n">
         <v>-25</v>
       </c>
-      <c r="M168" s="3" t="n">
+      <c r="M168" s="2" t="n">
         <v>-25</v>
       </c>
       <c r="N168" t="inlineStr">
@@ -9255,7 +9243,7 @@
       <c r="L169" t="n">
         <v>-29</v>
       </c>
-      <c r="M169" s="3" t="n">
+      <c r="M169" s="2" t="n">
         <v>-29</v>
       </c>
       <c r="N169" t="inlineStr">
@@ -9307,7 +9295,7 @@
       <c r="L170" t="n">
         <v>-29</v>
       </c>
-      <c r="M170" s="3" t="n">
+      <c r="M170" s="2" t="n">
         <v>-29</v>
       </c>
       <c r="N170" t="inlineStr">
@@ -9359,7 +9347,7 @@
       <c r="L171" t="n">
         <v>-29</v>
       </c>
-      <c r="M171" s="3" t="n">
+      <c r="M171" s="2" t="n">
         <v>-29</v>
       </c>
       <c r="N171" t="inlineStr">
@@ -9411,7 +9399,7 @@
       <c r="L172" t="n">
         <v>-37</v>
       </c>
-      <c r="M172" s="3" t="n">
+      <c r="M172" s="2" t="n">
         <v>-37</v>
       </c>
       <c r="N172" t="inlineStr">
@@ -9463,7 +9451,7 @@
       <c r="L173" t="n">
         <v>-38</v>
       </c>
-      <c r="M173" s="3" t="n">
+      <c r="M173" s="2" t="n">
         <v>-38</v>
       </c>
       <c r="N173" t="inlineStr">
@@ -9515,7 +9503,7 @@
       <c r="L174" t="n">
         <v>-38</v>
       </c>
-      <c r="M174" s="3" t="n">
+      <c r="M174" s="2" t="n">
         <v>-38</v>
       </c>
       <c r="N174" t="inlineStr">
@@ -9567,7 +9555,7 @@
       <c r="L175" t="n">
         <v>-40</v>
       </c>
-      <c r="M175" s="3" t="n">
+      <c r="M175" s="2" t="n">
         <v>-40</v>
       </c>
       <c r="N175" t="inlineStr">
@@ -9619,7 +9607,7 @@
       <c r="L176" t="n">
         <v>-40</v>
       </c>
-      <c r="M176" s="3" t="n">
+      <c r="M176" s="2" t="n">
         <v>-40</v>
       </c>
       <c r="N176" t="inlineStr">
@@ -9671,7 +9659,7 @@
       <c r="L177" t="n">
         <v>-45</v>
       </c>
-      <c r="M177" s="3" t="n">
+      <c r="M177" s="2" t="n">
         <v>-45</v>
       </c>
       <c r="N177" t="inlineStr">
@@ -9723,7 +9711,7 @@
       <c r="L178" t="n">
         <v>-68</v>
       </c>
-      <c r="M178" s="3" t="n">
+      <c r="M178" s="2" t="n">
         <v>-58</v>
       </c>
       <c r="N178" t="inlineStr">
@@ -9775,7 +9763,7 @@
       <c r="L179" t="n">
         <v>-67</v>
       </c>
-      <c r="M179" s="3" t="n">
+      <c r="M179" s="2" t="n">
         <v>-67</v>
       </c>
       <c r="N179" t="inlineStr">
@@ -9827,7 +9815,7 @@
       <c r="L180" t="n">
         <v>-67</v>
       </c>
-      <c r="M180" s="3" t="n">
+      <c r="M180" s="2" t="n">
         <v>-67</v>
       </c>
       <c r="N180" t="inlineStr">
@@ -9879,7 +9867,7 @@
       <c r="L181" t="n">
         <v>-207</v>
       </c>
-      <c r="M181" s="3" t="n">
+      <c r="M181" s="2" t="n">
         <v>-252</v>
       </c>
       <c r="N181" t="inlineStr">
@@ -9931,7 +9919,7 @@
       <c r="L182" t="n">
         <v>-1386</v>
       </c>
-      <c r="M182" s="3" t="n">
+      <c r="M182" s="2" t="n">
         <v>-1401</v>
       </c>
       <c r="N182" t="inlineStr">

</xml_diff>